<commit_message>
chore: atualiza planilhas de notas e gitignore
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/assets/notas/especial-2023.xlsx
+++ b/dashboard/assets/notas/especial-2023.xlsx
@@ -1,293 +1,42 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Planilhas</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>7</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="7" baseType="lpstr">
-      <vt:lpstr>TOTAL</vt:lpstr>
-      <vt:lpstr>COREOGRAFIA</vt:lpstr>
-      <vt:lpstr>MARCAÇÃO</vt:lpstr>
-      <vt:lpstr>ANIMAÇÃO</vt:lpstr>
-      <vt:lpstr>FIGURINO</vt:lpstr>
-      <vt:lpstr>CASAL DE NOIVOS</vt:lpstr>
-      <vt:lpstr>TRILHA SONORA</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
+  <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tiago\Documents\GitHub\site-linq-dfe-beta\dashboard\assets\notas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB6248B-D89F-42CE-B1CA-1167FD32F2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="TOTAL" sheetId="2" r:id="rId1"/>
+    <sheet name="COREOGRAFIA" sheetId="4" r:id="rId2"/>
+    <sheet name="MARCAÇÃO" sheetId="6" r:id="rId3"/>
+    <sheet name="ANIMAÇÃO" sheetId="8" r:id="rId4"/>
+    <sheet name="FIGURINO" sheetId="10" r:id="rId5"/>
+    <sheet name="CASAL DE NOIVOS" sheetId="12" r:id="rId6"/>
+    <sheet name="TRILHA SONORA" sheetId="14" r:id="rId7"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <cp:lastModifiedBy>Tiago</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-12T20:35:27Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-15T11:07:12Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="Created">
-    <vt:filetime>2026-02-02T00:00:00Z</vt:filetime>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="Creator">
-    <vt:lpwstr>www.smallpdf.com</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="LastSaved">
-    <vt:filetime>2026-03-12T00:00:00Z</vt:filetime>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="5" name="Producer">
-    <vt:lpwstr>www.smallpdf.com</vt:lpwstr>
-  </property>
-</Properties>
-</file>
-
-<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
-<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <c r="G16" i="14" l="1"/>
-  <c r="H16" i="14" s="1"/>
-  <c r="G15" i="14"/>
-  <c r="H15" i="14" s="1"/>
-  <c r="G14" i="14"/>
-  <c r="H14" i="14" s="1"/>
-  <c r="G13" i="14"/>
-  <c r="H13" i="14" s="1"/>
-  <c r="G12" i="14"/>
-  <c r="H12" i="14" s="1"/>
-  <c r="G11" i="14"/>
-  <c r="H11" i="14" s="1"/>
-  <c r="G10" i="14"/>
-  <c r="H10" i="14" s="1"/>
-  <c r="G9" i="14"/>
-  <c r="H9" i="14" s="1"/>
-  <c r="G8" i="14"/>
-  <c r="H8" i="14" s="1"/>
-  <c r="G7" i="14"/>
-  <c r="H7" i="14" s="1"/>
-  <c r="G6" i="14"/>
-  <c r="H6" i="14" s="1"/>
-  <c r="G5" i="14"/>
-  <c r="H5" i="14" s="1"/>
-  <c r="G4" i="14"/>
-  <c r="H4" i="14" s="1"/>
-  <c r="G3" i="14"/>
-  <c r="H3" i="14" s="1"/>
-  <c r="G2" i="14"/>
-  <c r="H2" i="14" s="1"/>
-  <c r="G16" i="12"/>
-  <c r="H16" i="12" s="1"/>
-  <c r="G15" i="12"/>
-  <c r="H15" i="12" s="1"/>
-  <c r="G14" i="12"/>
-  <c r="H14" i="12" s="1"/>
-  <c r="G13" i="12"/>
-  <c r="H13" i="12" s="1"/>
-  <c r="G12" i="12"/>
-  <c r="H12" i="12" s="1"/>
-  <c r="G11" i="12"/>
-  <c r="H11" i="12" s="1"/>
-  <c r="G10" i="12"/>
-  <c r="H10" i="12" s="1"/>
-  <c r="G9" i="12"/>
-  <c r="H9" i="12" s="1"/>
-  <c r="G8" i="12"/>
-  <c r="H8" i="12" s="1"/>
-  <c r="G7" i="12"/>
-  <c r="H7" i="12" s="1"/>
-  <c r="G6" i="12"/>
-  <c r="H6" i="12" s="1"/>
-  <c r="G5" i="12"/>
-  <c r="H5" i="12" s="1"/>
-  <c r="G4" i="12"/>
-  <c r="H4" i="12" s="1"/>
-  <c r="G3" i="12"/>
-  <c r="H3" i="12" s="1"/>
-  <c r="G2" i="12"/>
-  <c r="H2" i="12" s="1"/>
-  <c r="G16" i="10"/>
-  <c r="H16" i="10" s="1"/>
-  <c r="G15" i="10"/>
-  <c r="H15" i="10" s="1"/>
-  <c r="G14" i="10"/>
-  <c r="H14" i="10" s="1"/>
-  <c r="G13" i="10"/>
-  <c r="H13" i="10" s="1"/>
-  <c r="G12" i="10"/>
-  <c r="H12" i="10" s="1"/>
-  <c r="G11" i="10"/>
-  <c r="H11" i="10" s="1"/>
-  <c r="G10" i="10"/>
-  <c r="H10" i="10" s="1"/>
-  <c r="G9" i="10"/>
-  <c r="H9" i="10" s="1"/>
-  <c r="G8" i="10"/>
-  <c r="H8" i="10" s="1"/>
-  <c r="G7" i="10"/>
-  <c r="H7" i="10" s="1"/>
-  <c r="G6" i="10"/>
-  <c r="H6" i="10" s="1"/>
-  <c r="G5" i="10"/>
-  <c r="H5" i="10" s="1"/>
-  <c r="G4" i="10"/>
-  <c r="H4" i="10" s="1"/>
-  <c r="G3" i="10"/>
-  <c r="H3" i="10" s="1"/>
-  <c r="H2" i="10"/>
-  <c r="G2" i="10"/>
-  <c r="G16" i="8"/>
-  <c r="H16" i="8" s="1"/>
-  <c r="G15" i="8"/>
-  <c r="H15" i="8" s="1"/>
-  <c r="G14" i="8"/>
-  <c r="H14" i="8" s="1"/>
-  <c r="G13" i="8"/>
-  <c r="H13" i="8" s="1"/>
-  <c r="G12" i="8"/>
-  <c r="H12" i="8" s="1"/>
-  <c r="G11" i="8"/>
-  <c r="H11" i="8" s="1"/>
-  <c r="G10" i="8"/>
-  <c r="H10" i="8" s="1"/>
-  <c r="G9" i="8"/>
-  <c r="H9" i="8" s="1"/>
-  <c r="G8" i="8"/>
-  <c r="H8" i="8" s="1"/>
-  <c r="G7" i="8"/>
-  <c r="H7" i="8" s="1"/>
-  <c r="G6" i="8"/>
-  <c r="H6" i="8" s="1"/>
-  <c r="G5" i="8"/>
-  <c r="H5" i="8" s="1"/>
-  <c r="G4" i="8"/>
-  <c r="H4" i="8" s="1"/>
-  <c r="G3" i="8"/>
-  <c r="H3" i="8" s="1"/>
-  <c r="G2" i="8"/>
-  <c r="H2" i="8" s="1"/>
-  <c r="G16" i="6"/>
-  <c r="H16" i="6" s="1"/>
-  <c r="G15" i="6"/>
-  <c r="H15" i="6" s="1"/>
-  <c r="G14" i="6"/>
-  <c r="H14" i="6" s="1"/>
-  <c r="G13" i="6"/>
-  <c r="H13" i="6" s="1"/>
-  <c r="G12" i="6"/>
-  <c r="H12" i="6" s="1"/>
-  <c r="G11" i="6"/>
-  <c r="H11" i="6" s="1"/>
-  <c r="G10" i="6"/>
-  <c r="H10" i="6" s="1"/>
-  <c r="G9" i="6"/>
-  <c r="H9" i="6" s="1"/>
-  <c r="G8" i="6"/>
-  <c r="H8" i="6" s="1"/>
-  <c r="G7" i="6"/>
-  <c r="H7" i="6" s="1"/>
-  <c r="G6" i="6"/>
-  <c r="H6" i="6" s="1"/>
-  <c r="G5" i="6"/>
-  <c r="H5" i="6" s="1"/>
-  <c r="G4" i="6"/>
-  <c r="H4" i="6" s="1"/>
-  <c r="G3" i="6"/>
-  <c r="H3" i="6" s="1"/>
-  <c r="G2" i="6"/>
-  <c r="H2" i="6" s="1"/>
-  <c r="H3" i="4"/>
-  <c r="H4" i="4"/>
-  <c r="H5" i="4"/>
-  <c r="H6" i="4"/>
-  <c r="H7" i="4"/>
-  <c r="H8" i="4"/>
-  <c r="H9" i="4"/>
-  <c r="H10" i="4"/>
-  <c r="H11" i="4"/>
-  <c r="H12" i="4"/>
-  <c r="H13" i="4"/>
-  <c r="H14" i="4"/>
-  <c r="H15" i="4"/>
-  <c r="H16" i="4"/>
-  <c r="H2" i="4"/>
-  <c r="G3" i="4"/>
-  <c r="G4" i="4"/>
-  <c r="G5" i="4"/>
-  <c r="G6" i="4"/>
-  <c r="G7" i="4"/>
-  <c r="G8" i="4"/>
-  <c r="G9" i="4"/>
-  <c r="G10" i="4"/>
-  <c r="G11" i="4"/>
-  <c r="G12" i="4"/>
-  <c r="G13" i="4"/>
-  <c r="G14" i="4"/>
-  <c r="G15" i="4"/>
-  <c r="G16" i="4"/>
-  <c r="G2" i="4"/>
-  <c r="H2" i="2"/>
-  <c r="G2" i="2"/>
-  <c r="I2" i="2" s="1"/>
-  <c r="G10" i="2"/>
-  <c r="H10" i="2" s="1"/>
-  <c r="I10" i="2" s="1"/>
-  <c r="G3" i="2"/>
-  <c r="H3" i="2" s="1"/>
-  <c r="I3" i="2" s="1"/>
-  <c r="G4" i="2"/>
-  <c r="H4" i="2" s="1"/>
-  <c r="I4" i="2" s="1"/>
-  <c r="G5" i="2"/>
-  <c r="H5" i="2" s="1"/>
-  <c r="I5" i="2" s="1"/>
-  <c r="G6" i="2"/>
-  <c r="H6" i="2" s="1"/>
-  <c r="I6" i="2" s="1"/>
-  <c r="G7" i="2"/>
-  <c r="H7" i="2" s="1"/>
-  <c r="I7" i="2" s="1"/>
-  <c r="G8" i="2"/>
-  <c r="H8" i="2" s="1"/>
-  <c r="I8" i="2" s="1"/>
-  <c r="G9" i="2"/>
-  <c r="H9" i="2" s="1"/>
-  <c r="I9" i="2" s="1"/>
-  <c r="G11" i="2"/>
-  <c r="H11" i="2" s="1"/>
-  <c r="I11" i="2" s="1"/>
-  <c r="G12" i="2"/>
-  <c r="H12" i="2" s="1"/>
-  <c r="I12" i="2" s="1"/>
-  <c r="G13" i="2"/>
-  <c r="H13" i="2" s="1"/>
-  <c r="I13" i="2" s="1"/>
-  <c r="G14" i="2"/>
-  <c r="H14" i="2" s="1"/>
-  <c r="I14" i="2" s="1"/>
-  <c r="G15" i="2"/>
-  <c r="H15" i="2" s="1"/>
-  <c r="I15" i="2" s="1"/>
-  <c r="G16" i="2"/>
-  <c r="H16" i="2" s="1"/>
-  <c r="I16" i="2" s="1"/>
-</calcChain>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="46">
   <si>
     <r>
@@ -759,11 +508,10 @@
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -974,7 +722,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1074,9 +822,6 @@
     <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1094,7 +839,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1413,44 +1158,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tiago\Documents\GitHub\fantasy-junino\assets\notas\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291B92D2-4420-4577-AAF3-F6537914D10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="TOTAL" sheetId="2" r:id="rId1"/>
-    <sheet name="COREOGRAFIA" sheetId="4" r:id="rId2"/>
-    <sheet name="MARCAÇÃO" sheetId="6" r:id="rId3"/>
-    <sheet name="ANIMAÇÃO" sheetId="8" r:id="rId4"/>
-    <sheet name="FIGURINO" sheetId="10" r:id="rId5"/>
-    <sheet name="CASAL DE NOIVOS" sheetId="12" r:id="rId6"/>
-    <sheet name="TRILHA SONORA" sheetId="14" r:id="rId7"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -1503,13 +1211,16 @@
         <v>538.9</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>179.63333333333333</v>
       </c>
       <c r="H2">
-        <f>G2/6</f>
+        <f t="shared" ref="H2:H16" si="1">G2/6</f>
+        <v>29.938888888888886</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I16" si="2">H2/3</f>
+        <v>9.9796296296296294</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="13.7" customHeight="1">
@@ -1532,13 +1243,16 @@
         <v>538.20000000000005</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>179.4</v>
       </c>
       <c r="H3">
-        <f>G3/6</f>
+        <f t="shared" si="1"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="13.7" customHeight="1">
@@ -1561,13 +1275,16 @@
         <v>537.1</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>179.03333333333333</v>
       </c>
       <c r="H4">
-        <f>G4/6</f>
+        <f t="shared" si="1"/>
+        <v>29.838888888888889</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9462962962962962</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="13.7" customHeight="1">
@@ -1590,13 +1307,16 @@
         <v>535.29999999999995</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.43333333333331</v>
       </c>
       <c r="H5">
-        <f>G5/6</f>
+        <f t="shared" si="1"/>
+        <v>29.738888888888884</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9129629629629612</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="13.7" customHeight="1">
@@ -1619,13 +1339,16 @@
         <v>535.1</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.36666666666667</v>
       </c>
       <c r="H6">
-        <f>G6/6</f>
+        <f t="shared" si="1"/>
+        <v>29.727777777777778</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9092592592592599</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="13.7" customHeight="1">
@@ -1648,13 +1371,16 @@
         <v>534.79999999999995</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.26666666666665</v>
       </c>
       <c r="H7">
-        <f>G7/6</f>
+        <f t="shared" si="1"/>
+        <v>29.711111111111109</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9037037037037035</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="13.7" customHeight="1">
@@ -1677,13 +1403,16 @@
         <v>534.79999999999995</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.26666666666665</v>
       </c>
       <c r="H8">
-        <f>G8/6</f>
+        <f t="shared" si="1"/>
+        <v>29.711111111111109</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9037037037037035</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="13.7" customHeight="1">
@@ -1706,13 +1435,16 @@
         <v>534.6</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.20000000000002</v>
       </c>
       <c r="H9">
-        <f>G9/6</f>
+        <f t="shared" si="1"/>
+        <v>29.700000000000003</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="2"/>
+        <v>9.9</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="13.7" customHeight="1">
@@ -1735,13 +1467,16 @@
         <v>534.1</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>178.03333333333333</v>
       </c>
       <c r="H10">
-        <f>G10/6</f>
+        <f t="shared" si="1"/>
+        <v>29.672222222222221</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8907407407407408</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="13.7" customHeight="1">
@@ -1764,13 +1499,16 @@
         <v>532.70000000000005</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>177.56666666666669</v>
       </c>
       <c r="H11">
-        <f>G11/6</f>
+        <f t="shared" si="1"/>
+        <v>29.594444444444449</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8648148148148156</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="13.7" customHeight="1">
@@ -1793,13 +1531,16 @@
         <v>532.70000000000005</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>177.56666666666669</v>
       </c>
       <c r="H12">
-        <f>G12/6</f>
+        <f t="shared" si="1"/>
+        <v>29.594444444444449</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8648148148148156</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="13.7" customHeight="1">
@@ -1822,13 +1563,16 @@
         <v>532.29999999999995</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>177.43333333333331</v>
       </c>
       <c r="H13">
-        <f>G13/6</f>
+        <f t="shared" si="1"/>
+        <v>29.572222222222219</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8574074074074058</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="13.7" customHeight="1">
@@ -1851,13 +1595,16 @@
         <v>530.6</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>176.86666666666667</v>
       </c>
       <c r="H14">
-        <f>G14/6</f>
+        <f t="shared" si="1"/>
+        <v>29.477777777777778</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
+        <f t="shared" si="2"/>
+        <v>9.825925925925926</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="13.7" customHeight="1">
@@ -1880,13 +1627,16 @@
         <v>529.70000000000005</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>176.56666666666669</v>
       </c>
       <c r="H15">
-        <f>G15/6</f>
+        <f t="shared" si="1"/>
+        <v>29.427777777777781</v>
       </c>
       <c r="I15">
-        <f>H15/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8092592592592602</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="13.7" customHeight="1">
@@ -1909,13 +1659,16 @@
         <v>529.5</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>176.5</v>
       </c>
       <c r="H16">
-        <f>G16/6</f>
+        <f t="shared" si="1"/>
+        <v>29.416666666666668</v>
       </c>
       <c r="I16">
-        <f>H16/3</f>
+        <f t="shared" si="2"/>
+        <v>9.8055555555555554</v>
       </c>
     </row>
   </sheetData>
@@ -1924,7 +1677,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -1976,10 +1729,12 @@
         <v>89.5</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>29.833333333333332</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>9.9444444444444446</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -2002,10 +1757,12 @@
         <v>88.9</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -2028,10 +1785,12 @@
         <v>88.5</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.5</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8333333333333339</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -2054,10 +1813,12 @@
         <v>88.4</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.466666666666669</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8222222222222229</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -2080,10 +1841,12 @@
         <v>88.3</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.433333333333334</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8111111111111118</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -2106,10 +1869,12 @@
         <v>88.1</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.366666666666664</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7888888888888879</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -2132,10 +1897,12 @@
         <v>87.8</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.266666666666666</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7555555555555546</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -2158,10 +1925,12 @@
         <v>87.7</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.233333333333334</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7444444444444454</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -2184,10 +1953,12 @@
         <v>87.6</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.2</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7333333333333325</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -2210,10 +1981,12 @@
         <v>87.5</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.166666666666668</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7222222222222232</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -2234,10 +2007,12 @@
         <v>87.5</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.166666666666668</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7222222222222232</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -2260,10 +2035,12 @@
         <v>87.3</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.099999999999998</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -2286,10 +2063,12 @@
         <v>87.2</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.066666666666666</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6888888888888882</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -2312,10 +2091,12 @@
         <v>87.1</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.033333333333331</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6777777777777771</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -2338,10 +2119,12 @@
         <v>86.4</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.8</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6</v>
       </c>
     </row>
   </sheetData>
@@ -2353,7 +2136,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -2405,10 +2188,12 @@
         <v>89.8</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>29.933333333333334</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>9.9777777777777779</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -2431,10 +2216,12 @@
         <v>89.7</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -2457,10 +2244,12 @@
         <v>89.6</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -2483,10 +2272,12 @@
         <v>89.2</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.733333333333334</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9111111111111114</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -2509,10 +2300,12 @@
         <v>89.1</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.7</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -2533,10 +2326,12 @@
         <v>89.1</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.7</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -2559,10 +2354,12 @@
         <v>88.9</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -2583,10 +2380,12 @@
         <v>88.9</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -2609,10 +2408,12 @@
         <v>88.8</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.599999999999998</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666654</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -2635,10 +2436,12 @@
         <v>88.7</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.566666666666666</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8555555555555561</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -2661,10 +2464,12 @@
         <v>88.7</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.566666666666666</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8555555555555561</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -2687,10 +2492,12 @@
         <v>88.5</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.5</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8333333333333339</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -2713,10 +2520,12 @@
         <v>88.4</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.466666666666669</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8222222222222229</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -2739,10 +2548,12 @@
         <v>88.2</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.400000000000002</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8000000000000007</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -2765,10 +2576,12 @@
         <v>87.9</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.3</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7666666666666675</v>
       </c>
     </row>
   </sheetData>
@@ -2780,7 +2593,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -2832,10 +2645,12 @@
         <v>90</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>30</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -2856,10 +2671,12 @@
         <v>90</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -2882,10 +2699,12 @@
         <v>89.8</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.933333333333334</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9777777777777779</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -2908,10 +2727,12 @@
         <v>89.7</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -2932,10 +2753,12 @@
         <v>89.7</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -2958,10 +2781,12 @@
         <v>89.5</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.833333333333332</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9444444444444446</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -2984,10 +2809,12 @@
         <v>89.3</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.766666666666666</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9222222222222225</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -3008,10 +2835,12 @@
         <v>89.3</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.766666666666666</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9222222222222225</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -3034,10 +2863,12 @@
         <v>89</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.666666666666668</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8888888888888893</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -3058,10 +2889,12 @@
         <v>89</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.666666666666668</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8888888888888893</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -3084,10 +2917,12 @@
         <v>88.8</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.599999999999998</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666654</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -3108,10 +2943,12 @@
         <v>88.8</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.599999999999998</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666654</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -3134,10 +2971,12 @@
         <v>88.1</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.366666666666664</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7888888888888879</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -3160,10 +2999,12 @@
         <v>87.4</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.133333333333336</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7111111111111121</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -3186,10 +3027,12 @@
         <v>87.2</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.066666666666666</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6888888888888882</v>
       </c>
     </row>
   </sheetData>
@@ -3201,7 +3044,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -3253,10 +3096,12 @@
         <v>90</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>30</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -3277,10 +3122,12 @@
         <v>90</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -3303,10 +3150,12 @@
         <v>89.9</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -3327,10 +3176,12 @@
         <v>89.9</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -3351,10 +3202,12 @@
         <v>89.9</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -3377,10 +3230,12 @@
         <v>89.8</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.933333333333334</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9777777777777779</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -3403,10 +3258,12 @@
         <v>89.6</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -3427,10 +3284,12 @@
         <v>89.6</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -3451,10 +3310,12 @@
         <v>89.6</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -3477,10 +3338,12 @@
         <v>89.4</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -3501,10 +3364,12 @@
         <v>89.4</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -3525,10 +3390,12 @@
         <v>89.4</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -3551,10 +3418,12 @@
         <v>89.2</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.733333333333334</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9111111111111114</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -3575,10 +3444,12 @@
         <v>89.2</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.733333333333334</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9111111111111114</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -3601,10 +3472,12 @@
         <v>88.9</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
   </sheetData>
@@ -3616,7 +3489,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -3668,10 +3541,12 @@
         <v>90</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>30</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -3694,10 +3569,12 @@
         <v>89.8</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.933333333333334</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9777777777777779</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -3720,10 +3597,12 @@
         <v>89.7</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -3746,10 +3625,12 @@
         <v>89.5</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.833333333333332</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9444444444444446</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -3772,10 +3653,12 @@
         <v>89.5</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.833333333333332</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9444444444444446</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -3798,10 +3681,12 @@
         <v>89.4</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -3824,10 +3709,12 @@
         <v>89.3</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.766666666666666</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9222222222222225</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -3850,10 +3737,12 @@
         <v>89</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.666666666666668</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8888888888888893</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -3876,10 +3765,12 @@
         <v>88.9</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -3902,10 +3793,12 @@
         <v>88.9</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.633333333333336</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8777777777777782</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -3928,10 +3821,12 @@
         <v>88.8</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.599999999999998</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666654</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -3954,10 +3849,12 @@
         <v>88.3</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.433333333333334</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8111111111111118</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -3980,10 +3877,12 @@
         <v>88.2</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.400000000000002</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8000000000000007</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -4006,10 +3905,12 @@
         <v>87.7</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.233333333333334</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7444444444444454</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -4032,10 +3933,12 @@
         <v>87.6</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.2</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7333333333333325</v>
       </c>
     </row>
   </sheetData>
@@ -4047,7 +3950,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -4096,13 +3999,16 @@
         <v>30</v>
       </c>
       <c r="F2" s="5">
+        <f>SUM(C2:E2)</f>
         <v>90</v>
       </c>
       <c r="G2">
-        <f>F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <f t="shared" ref="G2:G16" si="0">F2/COUNTIF(C2:E2,"&lt;&gt;0")</f>
+        <v>30</v>
       </c>
       <c r="H2">
-        <f>G2/3</f>
+        <f t="shared" ref="H2:H16" si="1">G2/3</f>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
@@ -4119,14 +4025,17 @@
       <c r="E3" s="8">
         <v>30</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="5">
+        <f t="shared" ref="F3:F16" si="2">SUM(C3:E3)</f>
         <v>90</v>
       </c>
       <c r="G3">
-        <f>F3/COUNTIF(C3:E3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H3">
-        <f>G3/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1">
@@ -4143,14 +4052,17 @@
       <c r="E4" s="8">
         <v>30</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="5">
+        <f t="shared" si="2"/>
         <v>90</v>
       </c>
       <c r="G4">
-        <f>F4/COUNTIF(C4:E4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H4">
-        <f>G4/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1">
@@ -4167,14 +4079,17 @@
       <c r="E5" s="8">
         <v>30</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="5">
+        <f t="shared" si="2"/>
         <v>90</v>
       </c>
       <c r="G5">
-        <f>F5/COUNTIF(C5:E5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H5">
-        <f>G5/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1">
@@ -4191,14 +4106,17 @@
       <c r="E6" s="8">
         <v>30</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="5">
+        <f t="shared" si="2"/>
         <v>90</v>
       </c>
       <c r="G6">
-        <f>F6/COUNTIF(C6:E6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="H6">
-        <f>G6/3</f>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
@@ -4217,14 +4135,17 @@
       <c r="E7" s="8">
         <v>30</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="5">
+        <f t="shared" si="2"/>
         <v>89.9</v>
       </c>
       <c r="G7">
-        <f>F7/COUNTIF(C7:E7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H7">
-        <f>G7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1">
@@ -4241,14 +4162,17 @@
       <c r="E8" s="8">
         <v>30</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="5">
+        <f t="shared" si="2"/>
         <v>89.9</v>
       </c>
       <c r="G8">
-        <f>F8/COUNTIF(C8:E8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H8">
-        <f>G8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
@@ -4265,14 +4189,17 @@
       <c r="E9" s="8">
         <v>30</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="5">
+        <f t="shared" si="2"/>
         <v>89.9</v>
       </c>
       <c r="G9">
-        <f>F9/COUNTIF(C9:E9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H9">
-        <f>G9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
@@ -4289,14 +4216,17 @@
       <c r="E10" s="8">
         <v>30</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="5">
+        <f t="shared" si="2"/>
         <v>89.9</v>
       </c>
       <c r="G10">
-        <f>F10/COUNTIF(C10:E10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H10">
-        <f>G10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
@@ -4313,14 +4243,17 @@
       <c r="E11" s="8">
         <v>30</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="5">
+        <f t="shared" si="2"/>
         <v>89.9</v>
       </c>
       <c r="G11">
-        <f>F11/COUNTIF(C11:E11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.966666666666669</v>
       </c>
       <c r="H11">
-        <f>G11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9888888888888889</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
@@ -4339,14 +4272,17 @@
       <c r="E12" s="8">
         <v>30</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="5">
+        <f t="shared" si="2"/>
         <v>89.8</v>
       </c>
       <c r="G12">
-        <f>F12/COUNTIF(C12:E12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.933333333333334</v>
       </c>
       <c r="H12">
-        <f>G12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9777777777777779</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
@@ -4365,14 +4301,17 @@
       <c r="E13" s="8">
         <v>30</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="5">
+        <f t="shared" si="2"/>
         <v>89.7</v>
       </c>
       <c r="G13">
-        <f>F13/COUNTIF(C13:E13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.900000000000002</v>
       </c>
       <c r="H13">
-        <f>G13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9666666666666668</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
@@ -4391,14 +4330,17 @@
       <c r="E14" s="8">
         <v>30</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="5">
+        <f t="shared" si="2"/>
         <v>89.6</v>
       </c>
       <c r="G14">
-        <f>F14/COUNTIF(C14:E14,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H14">
-        <f>G14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
@@ -4415,14 +4357,17 @@
       <c r="E15" s="8">
         <v>30</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="5">
+        <f t="shared" si="2"/>
         <v>89.6</v>
       </c>
       <c r="G15">
-        <f>F15/COUNTIF(C15:E15,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.866666666666664</v>
       </c>
       <c r="H15">
-        <f>G15/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9555555555555539</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
@@ -4441,14 +4386,17 @@
       <c r="E16" s="8">
         <v>29.9</v>
       </c>
-      <c r="F16" s="9">
-        <v>89.2</v>
+      <c r="F16" s="5">
+        <f t="shared" si="2"/>
+        <v>89.199999999999989</v>
       </c>
       <c r="G16">
-        <f>F16/COUNTIF(C16:E16,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.733333333333331</v>
       </c>
       <c r="H16">
-        <f>G16/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9111111111111097</v>
       </c>
     </row>
   </sheetData>

</xml_diff>